<commit_message>
fix(capture): rebuild the workbook with holy-sheet 2.11.3 (column-index cell order)
The first build's rows were written A, AA, ..., B; Google Sheets dropped 184
input cells on import, so capture v1 computed over blanks. Same cases; new
bytes and digest.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/capture/v1/capture-v1.xlsx
+++ b/capture/v1/capture-v1.xlsx
@@ -13202,6 +13202,101 @@
       <c r="A1">
         <v>10</v>
       </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min_qty</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unit_price</t>
+        </is>
+      </c>
+      <c r="E1">
+        <v>30</v>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">apple</t>
+        </is>
+      </c>
+      <c r="H1">
+        <v>100</v>
+      </c>
+      <c r="I1">
+        <v>46307</v>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">=1+1</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d</t>
+        </is>
+      </c>
+      <c r="O1"/>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&gt;=200</t>
+        </is>
+      </c>
+      <c r="Q1">
+        <v>0.3</v>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">found</t>
+        </is>
+      </c>
+      <c r="S1">
+        <v>0</v>
+      </c>
+      <c r="T1">
+        <v>0</v>
+      </c>
+      <c r="U1">
+        <v>0</v>
+      </c>
+      <c r="V1">
+        <v>0.03</v>
+      </c>
+      <c r="W1">
+        <v>0</v>
+      </c>
+      <c r="X1">
+        <v>3</v>
+      </c>
+      <c r="Y1">
+        <v>5</v>
+      </c>
+      <c r="Z1">
+        <v>3</v>
+      </c>
       <c r="AA1">
         <v>3</v>
       </c>
@@ -13217,122 +13312,12 @@
       <c r="AE1">
         <v>5</v>
       </c>
-      <c r="B1">
-        <v>1</v>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">min_qty</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unit_price</t>
-        </is>
-      </c>
-      <c r="E1">
-        <v>30</v>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">c</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">apple</t>
-        </is>
-      </c>
-      <c r="H1">
-        <v>100</v>
-      </c>
-      <c r="I1">
-        <v>46307</v>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">=1+1</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">b</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">c</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d</t>
-        </is>
-      </c>
-      <c r="O1"/>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&gt;=200</t>
-        </is>
-      </c>
-      <c r="Q1">
-        <v>0.3</v>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">found</t>
-        </is>
-      </c>
-      <c r="S1">
-        <v>0</v>
-      </c>
-      <c r="T1">
-        <v>0</v>
-      </c>
-      <c r="U1">
-        <v>0</v>
-      </c>
-      <c r="V1">
-        <v>0.03</v>
-      </c>
-      <c r="W1">
-        <v>0</v>
-      </c>
-      <c r="X1">
-        <v>3</v>
-      </c>
-      <c r="Y1">
-        <v>5</v>
-      </c>
-      <c r="Z1">
-        <v>3</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">20</t>
         </is>
-      </c>
-      <c r="AA2" s="2">
-        <v>10</v>
-      </c>
-      <c r="AB2" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="2">
-        <v>30</v>
-      </c>
-      <c r="AD2" s="2">
-        <v>50</v>
-      </c>
-      <c r="AE2" s="2">
-        <v>200</v>
       </c>
       <c r="B2" s="2">
         <v>2</v>
@@ -13411,25 +13396,25 @@
       <c r="Z2" s="2">
         <v>24</v>
       </c>
+      <c r="AA2" s="2">
+        <v>10</v>
+      </c>
+      <c r="AB2" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="2">
+        <v>30</v>
+      </c>
+      <c r="AD2" s="2">
+        <v>50</v>
+      </c>
+      <c r="AE2" s="2">
+        <v>200</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="b">
         <v>1</v>
-      </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <v>5</v>
-      </c>
-      <c r="AC3">
-        <v>10</v>
-      </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
-      <c r="AE3">
-        <v>50</v>
       </c>
       <c r="B3">
         <v>3</v>
@@ -13498,24 +13483,24 @@
       <c r="Z3">
         <v>0</v>
       </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>5</v>
+      </c>
+      <c r="AC3">
+        <v>10</v>
+      </c>
+      <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>50</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2"/>
-      <c r="AA4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="2">
-        <v>0</v>
-      </c>
       <c r="B4" s="2">
         <v>4</v>
       </c>
@@ -13583,27 +13568,27 @@
       <c r="Z4" s="2">
         <v>0</v>
       </c>
+      <c r="AA4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t xml:space="preserve">abc</t>
         </is>
-      </c>
-      <c r="AA5">
-        <v>1000</v>
-      </c>
-      <c r="AB5">
-        <v>1000</v>
-      </c>
-      <c r="AC5">
-        <v>1000</v>
-      </c>
-      <c r="AD5">
-        <v>1000</v>
-      </c>
-      <c r="AE5">
-        <v>1000</v>
       </c>
       <c r="B5">
         <v>5</v>
@@ -13662,25 +13647,25 @@
       <c r="Z5">
         <v>1000</v>
       </c>
+      <c r="AA5">
+        <v>1000</v>
+      </c>
+      <c r="AB5">
+        <v>1000</v>
+      </c>
+      <c r="AC5">
+        <v>1000</v>
+      </c>
+      <c r="AD5">
+        <v>1000</v>
+      </c>
+      <c r="AE5">
+        <v>1000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
         <v>5</v>
-      </c>
-      <c r="AA6" s="2">
-        <v>400</v>
-      </c>
-      <c r="AB6" s="2">
-        <v>400</v>
-      </c>
-      <c r="AC6" s="2">
-        <v>400</v>
-      </c>
-      <c r="AD6" s="2">
-        <v>400</v>
-      </c>
-      <c r="AE6" s="2">
-        <v>400</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -13717,24 +13702,24 @@
       <c r="Z6" s="2">
         <v>400</v>
       </c>
+      <c r="AA6" s="2">
+        <v>400</v>
+      </c>
+      <c r="AB6" s="2">
+        <v>400</v>
+      </c>
+      <c r="AC6" s="2">
+        <v>400</v>
+      </c>
+      <c r="AD6" s="2">
+        <v>400</v>
+      </c>
+      <c r="AE6" s="2">
+        <v>400</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7"/>
-      <c r="AA7">
-        <v>600</v>
-      </c>
-      <c r="AB7">
-        <v>600</v>
-      </c>
-      <c r="AC7">
-        <v>600</v>
-      </c>
-      <c r="AD7">
-        <v>600</v>
-      </c>
-      <c r="AE7">
-        <v>600</v>
-      </c>
       <c r="B7"/>
       <c r="C7"/>
       <c r="D7"/>
@@ -13766,24 +13751,24 @@
       <c r="Z7">
         <v>600</v>
       </c>
+      <c r="AA7">
+        <v>600</v>
+      </c>
+      <c r="AB7">
+        <v>600</v>
+      </c>
+      <c r="AC7">
+        <v>600</v>
+      </c>
+      <c r="AD7">
+        <v>600</v>
+      </c>
+      <c r="AE7">
+        <v>600</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2"/>
-      <c r="AA8" s="2">
-        <v>1</v>
-      </c>
-      <c r="AB8" s="2">
-        <v>1</v>
-      </c>
-      <c r="AC8" s="2">
-        <v>9</v>
-      </c>
-      <c r="AD8" s="2">
-        <v>3</v>
-      </c>
-      <c r="AE8" s="2">
-        <v>5</v>
-      </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -13815,34 +13800,24 @@
       <c r="Z8" s="2">
         <v>1</v>
       </c>
+      <c r="AA8" s="2">
+        <v>1</v>
+      </c>
+      <c r="AB8" s="2">
+        <v>1</v>
+      </c>
+      <c r="AC8" s="2">
+        <v>9</v>
+      </c>
+      <c r="AD8" s="2">
+        <v>3</v>
+      </c>
+      <c r="AE8" s="2">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9"/>
-      <c r="AA9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">derived</t>
-        </is>
-      </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">entered</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">entered</t>
-        </is>
-      </c>
-      <c r="AD9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">entered</t>
-        </is>
-      </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">derived</t>
-        </is>
-      </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9"/>
@@ -13880,24 +13855,34 @@
           <t xml:space="preserve">entered</t>
         </is>
       </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">derived</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">entered</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">entered</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">entered</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">derived</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2"/>
-      <c r="AA10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AB10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AC10" s="2">
-        <v>200</v>
-      </c>
-      <c r="AD10" s="2">
-        <v>0</v>
-      </c>
-      <c r="AE10" s="2">
-        <v>0</v>
-      </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -13929,24 +13914,24 @@
       <c r="Z10" s="2">
         <v>0</v>
       </c>
+      <c r="AA10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="2">
+        <v>200</v>
+      </c>
+      <c r="AD10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE10" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11"/>
-      <c r="AA11">
-        <v>1</v>
-      </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
-      <c r="AC11">
-        <v>2</v>
-      </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
-      <c r="AE11">
-        <v>3</v>
-      </c>
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11"/>
@@ -13978,24 +13963,24 @@
       <c r="Z11">
         <v>0</v>
       </c>
+      <c r="AA11">
+        <v>1</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <v>2</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2"/>
-      <c r="AA12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AB12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD12" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE12" s="2" t="b">
-        <v>1</v>
-      </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -14027,24 +14012,24 @@
       <c r="Z12" s="2" t="b">
         <v>0</v>
       </c>
+      <c r="AA12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE12" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13"/>
-      <c r="AA13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AD13" t="b">
-        <v>0</v>
-      </c>
-      <c r="AE13" t="b">
-        <v>1</v>
-      </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13"/>
@@ -14076,6 +14061,21 @@
       <c r="Z13" t="b">
         <v>0</v>
       </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AE13" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>